<commit_message>
feat: add Papers page with S2T Chinese conversion
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a1234/Desktop/HK_UpUp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D0B8CA-67AC-6C40-9D1F-0A41F647E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DABCC589-9088-384A-B41B-CB3517DD01F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17300" xr2:uid="{0F542A8C-4579-B142-B085-8E1ABFA2FFAF}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17300" activeTab="1" xr2:uid="{0F542A8C-4579-B142-B085-8E1ABFA2FFAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Competitions" sheetId="1" r:id="rId1"/>
+    <sheet name="Papers" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -78,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>title</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -117,10 +118,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Certification</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://panpearl.iproa.org/web/</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -149,10 +146,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Certification, Internship opportunity</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://alipayhkadvice.seedfoundation.hk/uni/en/</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -162,6 +155,94 @@
   </si>
   <si>
     <t>AlipayHK, SEED Foundation, The Hong Kong Federation of Youth Groups</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Conference Full Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Official Website</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Conference Venue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Organizer</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027年第一届现代学习与教育技术国际会议</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Abbreviated Conference Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MLET 2027</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://mlet.net/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027年8月8-10日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日本·大阪</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Conference Dates</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日本大阪大学</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Registration Deadline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027年工程系统人工智能国际会议（ICAIES 2027）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ICAIES 2027</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>巴西里约热内卢</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027年3月5–7日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.icaies.org/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>India International Congress on Computational Intelligence (IICCI)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TBC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Certification, Internship opportunity, TBC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Certification, TBC</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -220,7 +301,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -235,6 +316,9 @@
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -726,7 +810,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C2" s="4">
         <v>46167</v>
@@ -735,10 +819,10 @@
         <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="G2" t="e" vm="1">
         <v>#VALUE!</v>
@@ -746,22 +830,22 @@
     </row>
     <row r="3" spans="1:7" ht="32">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="4">
         <v>46167</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3" s="3" t="e" vm="2">
         <v>#VALUE!</v>
@@ -769,22 +853,22 @@
     </row>
     <row r="4" spans="1:7" ht="96">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4">
         <v>46132</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="G4" s="3" t="e" vm="3">
         <v>#VALUE!</v>
@@ -802,4 +886,97 @@
     <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8B3420-51B2-1948-9322-8EFBB751BA0C}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{A5728AB0-BF91-554F-BA65-2B5EF4375A6A}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{DBBA7773-8480-C443-B224-6300A3030E0E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>